<commit_message>
translated model parameter units to English
</commit_message>
<xml_diff>
--- a/meal protein drink.xlsx
+++ b/meal protein drink.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27263E4E-DDF2-475C-B270-41BE11142DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
@@ -519,7 +519,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="meal"/>

</xml_diff>